<commit_message>
Audit SWCNT_synthetic_5000 dataset & PyKAN forward evaluation: clamp sensor noise to process bounds and export complete ground truth matrix
</commit_message>
<xml_diff>
--- a/nopo_paper_pkg/SWCNT_synthetic_50_matched.xlsx
+++ b/nopo_paper_pkg/SWCNT_synthetic_50_matched.xlsx
@@ -1041,6 +1041,9 @@
       <c r="T7">
         <v>14.46050035987868</v>
       </c>
+      <c r="U7">
+        <v>35.5309132359022</v>
+      </c>
       <c r="V7">
         <v>1004.993718122912</v>
       </c>
@@ -1676,7 +1679,7 @@
         <v>44.51121238793917</v>
       </c>
       <c r="D15">
-        <v>99.82535235945767</v>
+        <v>100</v>
       </c>
       <c r="E15">
         <v>10</v>
@@ -2239,6 +2242,9 @@
       <c r="S21">
         <v>1.290948930318683</v>
       </c>
+      <c r="T21">
+        <v>16.35439811422098</v>
+      </c>
       <c r="U21">
         <v>42.9287145880894</v>
       </c>
@@ -2411,6 +2417,9 @@
       <c r="T23">
         <v>14.10180916498922</v>
       </c>
+      <c r="U23">
+        <v>31.20794275047204</v>
+      </c>
       <c r="V23">
         <v>1089.344792564146</v>
       </c>
@@ -3096,6 +3105,9 @@
       <c r="T31">
         <v>10.48510458133969</v>
       </c>
+      <c r="U31">
+        <v>32.62355596843382</v>
+      </c>
       <c r="V31">
         <v>671.7957571390923</v>
       </c>
@@ -3265,6 +3277,9 @@
       <c r="T33">
         <v>17.17163252997251</v>
       </c>
+      <c r="U33">
+        <v>45.2896817469816</v>
+      </c>
       <c r="V33">
         <v>1315.838136582657</v>
       </c>
@@ -3348,6 +3363,27 @@
       <c r="T34">
         <v>16.71356927122181</v>
       </c>
+      <c r="U34">
+        <v>49.13109399038201</v>
+      </c>
+      <c r="V34">
+        <v>1498.974145334406</v>
+      </c>
+      <c r="W34">
+        <v>1500.949874784279</v>
+      </c>
+      <c r="X34">
+        <v>341827.4047550822</v>
+      </c>
+      <c r="Y34">
+        <v>333070.5888323828</v>
+      </c>
+      <c r="Z34">
+        <v>1707.482527571321</v>
+      </c>
+      <c r="AA34">
+        <v>1703.57583858049</v>
+      </c>
       <c r="AB34" t="s">
         <v>28</v>
       </c>
@@ -3585,6 +3621,9 @@
       <c r="T37">
         <v>16.59668273886943</v>
       </c>
+      <c r="U37">
+        <v>43.84966027261194</v>
+      </c>
       <c r="V37">
         <v>1172.250837272215</v>
       </c>
@@ -3751,6 +3790,9 @@
       <c r="S39">
         <v>0.493991083411384</v>
       </c>
+      <c r="T39">
+        <v>13.16110393966917</v>
+      </c>
       <c r="U39">
         <v>34.29029190873455</v>
       </c>
@@ -3840,6 +3882,24 @@
       <c r="U40">
         <v>40.95279972095296</v>
       </c>
+      <c r="V40">
+        <v>1182.617093819365</v>
+      </c>
+      <c r="W40">
+        <v>1236.182731142273</v>
+      </c>
+      <c r="X40">
+        <v>300444.2595668557</v>
+      </c>
+      <c r="Y40">
+        <v>288907.8222843089</v>
+      </c>
+      <c r="Z40">
+        <v>1168.434289335146</v>
+      </c>
+      <c r="AA40">
+        <v>1143.62827628378</v>
+      </c>
       <c r="AB40" t="s">
         <v>28</v>
       </c>
@@ -4080,6 +4140,24 @@
       <c r="U43">
         <v>39.57596118817513</v>
       </c>
+      <c r="V43">
+        <v>1157.606813983687</v>
+      </c>
+      <c r="W43">
+        <v>1100.305583743807</v>
+      </c>
+      <c r="X43">
+        <v>268154.1125776102</v>
+      </c>
+      <c r="Y43">
+        <v>259030.1528970982</v>
+      </c>
+      <c r="Z43">
+        <v>1322.944108752529</v>
+      </c>
+      <c r="AA43">
+        <v>1284.274648052572</v>
+      </c>
       <c r="AB43" t="s">
         <v>28</v>
       </c>
@@ -4181,7 +4259,7 @@
         <v>80</v>
       </c>
       <c r="D45">
-        <v>99.32897809310828</v>
+        <v>100</v>
       </c>
       <c r="E45">
         <v>10</v>
@@ -4314,6 +4392,9 @@
       <c r="S46">
         <v>1.946036363781111</v>
       </c>
+      <c r="T46">
+        <v>18.24728856439808</v>
+      </c>
       <c r="U46">
         <v>45.61383247083607</v>
       </c>
@@ -4572,6 +4653,27 @@
       <c r="T49">
         <v>17.94872434551969</v>
       </c>
+      <c r="U49">
+        <v>44.56800078096127</v>
+      </c>
+      <c r="V49">
+        <v>1395.06700512197</v>
+      </c>
+      <c r="W49">
+        <v>1399.090321464704</v>
+      </c>
+      <c r="X49">
+        <v>307505.7466545154</v>
+      </c>
+      <c r="Y49">
+        <v>303569.9101591521</v>
+      </c>
+      <c r="Z49">
+        <v>1139.682386602218</v>
+      </c>
+      <c r="AA49">
+        <v>1098.650574507692</v>
+      </c>
       <c r="AB49" t="s">
         <v>28</v>
       </c>
@@ -4725,6 +4827,24 @@
       </c>
       <c r="U51">
         <v>37.99453191006525</v>
+      </c>
+      <c r="V51">
+        <v>1131.735391473701</v>
+      </c>
+      <c r="W51">
+        <v>1160.328852827805</v>
+      </c>
+      <c r="X51">
+        <v>262536.7285192074</v>
+      </c>
+      <c r="Y51">
+        <v>252866.4906258908</v>
+      </c>
+      <c r="Z51">
+        <v>1231.742621787504</v>
+      </c>
+      <c r="AA51">
+        <v>1264.41018765091</v>
       </c>
       <c r="AB51" t="s">
         <v>28</v>

</xml_diff>